<commit_message>
Fixed the error of printing out Onboard Equipment, Redesigned the Train Availability and Incident Summary Report, and Regressed Clearance Form because of error
</commit_message>
<xml_diff>
--- a/forms/TAR_template.xlsx
+++ b/forms/TAR_template.xlsx
@@ -972,46 +972,46 @@
       <c r="A1" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="R1" s="52" t="n"/>
-      <c r="S1" s="52" t="n"/>
-      <c r="T1" s="52" t="n"/>
-      <c r="U1" s="52" t="n"/>
+      <c r="R1" s="52"/>
+      <c r="S1" s="52"/>
+      <c r="T1" s="52"/>
+      <c r="U1" s="52"/>
     </row>
     <row r="2" ht="14.4" customHeight="1" s="50">
       <c r="A2" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="R2" s="54" t="n"/>
-      <c r="S2" s="54" t="n"/>
-      <c r="T2" s="54" t="n"/>
-      <c r="U2" s="54" t="n"/>
+      <c r="R2" s="54"/>
+      <c r="S2" s="54"/>
+      <c r="T2" s="54"/>
+      <c r="U2" s="54"/>
     </row>
     <row r="3" ht="14.4" customHeight="1" s="50">
       <c r="A3" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="R3" s="54" t="n"/>
-      <c r="S3" s="54" t="n"/>
-      <c r="T3" s="54" t="n"/>
-      <c r="U3" s="54" t="n"/>
+      <c r="R3" s="54"/>
+      <c r="S3" s="54"/>
+      <c r="T3" s="54"/>
+      <c r="U3" s="54"/>
     </row>
     <row r="4" ht="14.4" customHeight="1" s="50">
       <c r="A4" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="R4" s="54" t="n"/>
-      <c r="S4" s="54" t="n"/>
-      <c r="T4" s="54" t="n"/>
-      <c r="U4" s="54" t="n"/>
+      <c r="R4" s="54"/>
+      <c r="S4" s="54"/>
+      <c r="T4" s="54"/>
+      <c r="U4" s="54"/>
     </row>
     <row r="6" ht="18" customHeight="1" s="50">
       <c r="A6" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="R6" s="56" t="n"/>
-      <c r="S6" s="56" t="n"/>
-      <c r="T6" s="56" t="n"/>
-      <c r="U6" s="56" t="n"/>
+      <c r="R6" s="56"/>
+      <c r="S6" s="56"/>
+      <c r="T6" s="56"/>
+      <c r="U6" s="56"/>
     </row>
     <row r="8" ht="13.8" customFormat="1" customHeight="1" s="57">
       <c r="A8" s="58" t="s">
@@ -1020,8 +1020,8 @@
       <c r="C8" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="58" t="n"/>
-      <c r="E8" s="58" t="n"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="58"/>
       <c r="I8" s="60" t="s">
         <v>7</v>
       </c>
@@ -1053,7 +1053,7 @@
       <c r="N10" s="61" t="s">
         <v>14</v>
       </c>
-      <c r="O10" s="62" t="n"/>
+      <c r="O10" s="62"/>
     </row>
     <row r="11" ht="14.4" customHeight="1" s="50"/>
     <row r="12" ht="27.75" customFormat="1" customHeight="1" s="63">
@@ -1093,30 +1093,30 @@
       <c r="L12" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="M12" s="69" t="n"/>
-      <c r="N12" s="69" t="n"/>
-      <c r="O12" s="70" t="n"/>
+      <c r="M12" s="69"/>
+      <c r="N12" s="69"/>
+      <c r="O12" s="70"/>
       <c r="P12" s="71" t="s">
         <v>22</v>
       </c>
-      <c r="Q12" s="72" t="n"/>
+      <c r="Q12" s="72"/>
     </row>
     <row r="13" ht="16.5" customFormat="1" customHeight="1" s="63">
-      <c r="A13" s="73" t="n"/>
-      <c r="B13" s="74" t="n"/>
-      <c r="C13" s="74" t="n"/>
-      <c r="D13" s="74" t="n"/>
-      <c r="E13" s="74" t="n"/>
-      <c r="F13" s="74" t="n"/>
-      <c r="G13" s="74" t="n"/>
-      <c r="H13" s="75" t="n"/>
-      <c r="I13" s="74" t="n"/>
-      <c r="J13" s="74" t="n"/>
-      <c r="K13" s="74" t="n"/>
-      <c r="L13" s="76" t="n"/>
-      <c r="M13" s="77" t="n"/>
-      <c r="N13" s="77" t="n"/>
-      <c r="O13" s="75" t="n"/>
+      <c r="A13" s="73"/>
+      <c r="B13" s="74"/>
+      <c r="C13" s="74"/>
+      <c r="D13" s="74"/>
+      <c r="E13" s="74"/>
+      <c r="F13" s="74"/>
+      <c r="G13" s="74"/>
+      <c r="H13" s="75"/>
+      <c r="I13" s="74"/>
+      <c r="J13" s="74"/>
+      <c r="K13" s="74"/>
+      <c r="L13" s="76"/>
+      <c r="M13" s="77"/>
+      <c r="N13" s="77"/>
+      <c r="O13" s="75"/>
       <c r="P13" s="78" t="s">
         <v>23</v>
       </c>
@@ -1125,574 +1125,574 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="50">
-      <c r="A14" s="80" t="n"/>
-      <c r="B14" s="80" t="n"/>
-      <c r="C14" s="80" t="n"/>
-      <c r="D14" s="80" t="n"/>
-      <c r="E14" s="80" t="n"/>
-      <c r="F14" s="80" t="n"/>
-      <c r="G14" s="80" t="n"/>
-      <c r="H14" s="81" t="n"/>
-      <c r="I14" s="81" t="n"/>
-      <c r="J14" s="81" t="n"/>
-      <c r="K14" s="81" t="n"/>
-      <c r="L14" s="82" t="n"/>
-      <c r="M14" s="83" t="n"/>
-      <c r="N14" s="83" t="n"/>
-      <c r="O14" s="83" t="n"/>
-      <c r="P14" s="84" t="n"/>
-      <c r="Q14" s="84" t="n"/>
+      <c r="A14" s="80"/>
+      <c r="B14" s="80"/>
+      <c r="C14" s="80"/>
+      <c r="D14" s="80"/>
+      <c r="E14" s="80"/>
+      <c r="F14" s="80"/>
+      <c r="G14" s="80"/>
+      <c r="H14" s="81"/>
+      <c r="I14" s="81"/>
+      <c r="J14" s="81"/>
+      <c r="K14" s="81"/>
+      <c r="L14" s="82"/>
+      <c r="M14" s="83"/>
+      <c r="N14" s="83"/>
+      <c r="O14" s="83"/>
+      <c r="P14" s="84"/>
+      <c r="Q14" s="84"/>
     </row>
     <row r="15" ht="7.5" customHeight="1" s="50">
-      <c r="A15" s="85" t="n"/>
-      <c r="B15" s="86" t="n"/>
-      <c r="C15" s="86" t="n"/>
-      <c r="D15" s="86" t="n"/>
-      <c r="E15" s="86" t="n"/>
-      <c r="F15" s="87" t="n"/>
-      <c r="G15" s="85" t="n"/>
-      <c r="H15" s="88" t="n"/>
-      <c r="I15" s="88" t="n"/>
-      <c r="J15" s="88" t="n"/>
-      <c r="K15" s="88" t="n"/>
-      <c r="L15" s="89" t="n"/>
-      <c r="M15" s="90" t="n"/>
-      <c r="N15" s="90" t="n"/>
-      <c r="O15" s="90" t="n"/>
-      <c r="P15" s="85" t="n"/>
-      <c r="Q15" s="85" t="n"/>
+      <c r="A15" s="85"/>
+      <c r="B15" s="86"/>
+      <c r="C15" s="86"/>
+      <c r="D15" s="86"/>
+      <c r="E15" s="86"/>
+      <c r="F15" s="87"/>
+      <c r="G15" s="85"/>
+      <c r="H15" s="88"/>
+      <c r="I15" s="88"/>
+      <c r="J15" s="88"/>
+      <c r="K15" s="88"/>
+      <c r="L15" s="89"/>
+      <c r="M15" s="90"/>
+      <c r="N15" s="90"/>
+      <c r="O15" s="90"/>
+      <c r="P15" s="85"/>
+      <c r="Q15" s="85"/>
     </row>
     <row r="16" ht="7.5" customHeight="1" s="50">
-      <c r="A16" s="85" t="n"/>
-      <c r="B16" s="87" t="n"/>
-      <c r="C16" s="87" t="n"/>
-      <c r="D16" s="87" t="n"/>
-      <c r="E16" s="87" t="n"/>
-      <c r="F16" s="86" t="n"/>
-      <c r="G16" s="85" t="n"/>
-      <c r="H16" s="88" t="n"/>
-      <c r="I16" s="88" t="n"/>
-      <c r="J16" s="88" t="n"/>
-      <c r="K16" s="88" t="n"/>
-      <c r="L16" s="89" t="n"/>
-      <c r="M16" s="90" t="n"/>
-      <c r="N16" s="90" t="n"/>
-      <c r="O16" s="90" t="n"/>
-      <c r="P16" s="85" t="n"/>
-      <c r="Q16" s="85" t="n"/>
+      <c r="A16" s="85"/>
+      <c r="B16" s="87"/>
+      <c r="C16" s="87"/>
+      <c r="D16" s="87"/>
+      <c r="E16" s="87"/>
+      <c r="F16" s="86"/>
+      <c r="G16" s="85"/>
+      <c r="H16" s="88"/>
+      <c r="I16" s="88"/>
+      <c r="J16" s="88"/>
+      <c r="K16" s="88"/>
+      <c r="L16" s="89"/>
+      <c r="M16" s="90"/>
+      <c r="N16" s="90"/>
+      <c r="O16" s="90"/>
+      <c r="P16" s="85"/>
+      <c r="Q16" s="85"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="50">
-      <c r="A17" s="86" t="n"/>
-      <c r="B17" s="86" t="n"/>
-      <c r="C17" s="86" t="n"/>
-      <c r="D17" s="86" t="n"/>
-      <c r="E17" s="86" t="n"/>
-      <c r="F17" s="87" t="n"/>
-      <c r="G17" s="86" t="n"/>
-      <c r="H17" s="91" t="n"/>
-      <c r="I17" s="91" t="n"/>
-      <c r="J17" s="91" t="n"/>
-      <c r="K17" s="91" t="n"/>
-      <c r="L17" s="92" t="n"/>
-      <c r="M17" s="93" t="n"/>
-      <c r="N17" s="93" t="n"/>
-      <c r="O17" s="93" t="n"/>
-      <c r="P17" s="86" t="n"/>
-      <c r="Q17" s="86" t="n"/>
+      <c r="A17" s="86"/>
+      <c r="B17" s="86"/>
+      <c r="C17" s="86"/>
+      <c r="D17" s="86"/>
+      <c r="E17" s="86"/>
+      <c r="F17" s="87"/>
+      <c r="G17" s="86"/>
+      <c r="H17" s="91"/>
+      <c r="I17" s="91"/>
+      <c r="J17" s="91"/>
+      <c r="K17" s="91"/>
+      <c r="L17" s="92"/>
+      <c r="M17" s="93"/>
+      <c r="N17" s="93"/>
+      <c r="O17" s="93"/>
+      <c r="P17" s="86"/>
+      <c r="Q17" s="86"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="50">
-      <c r="A18" s="94" t="n"/>
-      <c r="B18" s="94" t="n"/>
-      <c r="C18" s="94" t="n"/>
-      <c r="D18" s="94" t="n"/>
-      <c r="E18" s="94" t="n"/>
-      <c r="F18" s="94" t="n"/>
-      <c r="G18" s="87" t="n"/>
-      <c r="H18" s="95" t="n"/>
-      <c r="I18" s="95" t="n"/>
-      <c r="J18" s="95" t="n"/>
-      <c r="K18" s="95" t="n"/>
-      <c r="L18" s="96" t="n"/>
-      <c r="M18" s="97" t="n"/>
-      <c r="N18" s="97" t="n"/>
-      <c r="O18" s="97" t="n"/>
-      <c r="P18" s="98" t="n"/>
-      <c r="Q18" s="98" t="n"/>
+      <c r="A18" s="94"/>
+      <c r="B18" s="94"/>
+      <c r="C18" s="94"/>
+      <c r="D18" s="94"/>
+      <c r="E18" s="94"/>
+      <c r="F18" s="94"/>
+      <c r="G18" s="87"/>
+      <c r="H18" s="95"/>
+      <c r="I18" s="95"/>
+      <c r="J18" s="95"/>
+      <c r="K18" s="95"/>
+      <c r="L18" s="96"/>
+      <c r="M18" s="97"/>
+      <c r="N18" s="97"/>
+      <c r="O18" s="97"/>
+      <c r="P18" s="98"/>
+      <c r="Q18" s="98"/>
     </row>
     <row r="19" ht="7.5" customHeight="1" s="50">
-      <c r="A19" s="85" t="n"/>
-      <c r="B19" s="86" t="n"/>
-      <c r="C19" s="86" t="n"/>
-      <c r="D19" s="86" t="n"/>
-      <c r="E19" s="86" t="n"/>
-      <c r="F19" s="87" t="n"/>
-      <c r="G19" s="85" t="n"/>
-      <c r="H19" s="88" t="n"/>
-      <c r="I19" s="88" t="n"/>
-      <c r="J19" s="88" t="n"/>
-      <c r="K19" s="88" t="n"/>
-      <c r="L19" s="89" t="n"/>
-      <c r="M19" s="90" t="n"/>
-      <c r="N19" s="90" t="n"/>
-      <c r="O19" s="90" t="n"/>
-      <c r="P19" s="85" t="n"/>
-      <c r="Q19" s="85" t="n"/>
+      <c r="A19" s="85"/>
+      <c r="B19" s="86"/>
+      <c r="C19" s="86"/>
+      <c r="D19" s="86"/>
+      <c r="E19" s="86"/>
+      <c r="F19" s="87"/>
+      <c r="G19" s="85"/>
+      <c r="H19" s="88"/>
+      <c r="I19" s="88"/>
+      <c r="J19" s="88"/>
+      <c r="K19" s="88"/>
+      <c r="L19" s="89"/>
+      <c r="M19" s="90"/>
+      <c r="N19" s="90"/>
+      <c r="O19" s="90"/>
+      <c r="P19" s="85"/>
+      <c r="Q19" s="85"/>
     </row>
     <row r="20" ht="7.5" customHeight="1" s="50">
-      <c r="A20" s="85" t="n"/>
-      <c r="B20" s="87" t="n"/>
-      <c r="C20" s="87" t="n"/>
-      <c r="D20" s="87" t="n"/>
-      <c r="E20" s="87" t="n"/>
-      <c r="F20" s="86" t="n"/>
-      <c r="G20" s="85" t="n"/>
-      <c r="H20" s="88" t="n"/>
-      <c r="I20" s="88" t="n"/>
-      <c r="J20" s="88" t="n"/>
-      <c r="K20" s="88" t="n"/>
-      <c r="L20" s="89" t="n"/>
-      <c r="M20" s="90" t="n"/>
-      <c r="N20" s="90" t="n"/>
-      <c r="O20" s="90" t="n"/>
-      <c r="P20" s="85" t="n"/>
-      <c r="Q20" s="85" t="n"/>
+      <c r="A20" s="85"/>
+      <c r="B20" s="87"/>
+      <c r="C20" s="87"/>
+      <c r="D20" s="87"/>
+      <c r="E20" s="87"/>
+      <c r="F20" s="86"/>
+      <c r="G20" s="85"/>
+      <c r="H20" s="88"/>
+      <c r="I20" s="88"/>
+      <c r="J20" s="88"/>
+      <c r="K20" s="88"/>
+      <c r="L20" s="89"/>
+      <c r="M20" s="90"/>
+      <c r="N20" s="90"/>
+      <c r="O20" s="90"/>
+      <c r="P20" s="85"/>
+      <c r="Q20" s="85"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="50">
-      <c r="A21" s="86" t="n"/>
-      <c r="B21" s="86" t="n"/>
-      <c r="C21" s="86" t="n"/>
-      <c r="D21" s="86" t="n"/>
-      <c r="E21" s="86" t="n"/>
-      <c r="F21" s="87" t="n"/>
-      <c r="G21" s="86" t="n"/>
-      <c r="H21" s="91" t="n"/>
-      <c r="I21" s="91" t="n"/>
-      <c r="J21" s="91" t="n"/>
-      <c r="K21" s="91" t="n"/>
-      <c r="L21" s="92" t="n"/>
-      <c r="M21" s="93" t="n"/>
-      <c r="N21" s="93" t="n"/>
-      <c r="O21" s="93" t="n"/>
-      <c r="P21" s="86" t="n"/>
-      <c r="Q21" s="86" t="n"/>
+      <c r="A21" s="86"/>
+      <c r="B21" s="86"/>
+      <c r="C21" s="86"/>
+      <c r="D21" s="86"/>
+      <c r="E21" s="86"/>
+      <c r="F21" s="87"/>
+      <c r="G21" s="86"/>
+      <c r="H21" s="91"/>
+      <c r="I21" s="91"/>
+      <c r="J21" s="91"/>
+      <c r="K21" s="91"/>
+      <c r="L21" s="92"/>
+      <c r="M21" s="93"/>
+      <c r="N21" s="93"/>
+      <c r="O21" s="93"/>
+      <c r="P21" s="86"/>
+      <c r="Q21" s="86"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="50">
-      <c r="A22" s="94" t="n"/>
-      <c r="B22" s="94" t="n"/>
-      <c r="C22" s="94" t="n"/>
-      <c r="D22" s="94" t="n"/>
-      <c r="E22" s="94" t="n"/>
-      <c r="F22" s="94" t="n"/>
-      <c r="G22" s="87" t="n"/>
-      <c r="H22" s="99" t="n"/>
-      <c r="I22" s="99" t="n"/>
-      <c r="J22" s="99" t="n"/>
-      <c r="K22" s="99" t="n"/>
-      <c r="L22" s="96" t="n"/>
-      <c r="M22" s="97" t="n"/>
-      <c r="N22" s="97" t="n"/>
-      <c r="O22" s="97" t="n"/>
-      <c r="P22" s="98" t="n"/>
-      <c r="Q22" s="98" t="n"/>
+      <c r="A22" s="94"/>
+      <c r="B22" s="94"/>
+      <c r="C22" s="94"/>
+      <c r="D22" s="94"/>
+      <c r="E22" s="94"/>
+      <c r="F22" s="94"/>
+      <c r="G22" s="87"/>
+      <c r="H22" s="99"/>
+      <c r="I22" s="99"/>
+      <c r="J22" s="99"/>
+      <c r="K22" s="99"/>
+      <c r="L22" s="96"/>
+      <c r="M22" s="97"/>
+      <c r="N22" s="97"/>
+      <c r="O22" s="97"/>
+      <c r="P22" s="98"/>
+      <c r="Q22" s="98"/>
     </row>
     <row r="23" ht="7.5" customHeight="1" s="50">
-      <c r="A23" s="85" t="n"/>
-      <c r="B23" s="86" t="n"/>
-      <c r="C23" s="86" t="n"/>
-      <c r="D23" s="86" t="n"/>
-      <c r="E23" s="86" t="n"/>
-      <c r="F23" s="87" t="n"/>
-      <c r="G23" s="85" t="n"/>
-      <c r="H23" s="88" t="n"/>
-      <c r="I23" s="88" t="n"/>
-      <c r="J23" s="88" t="n"/>
-      <c r="K23" s="88" t="n"/>
-      <c r="L23" s="89" t="n"/>
-      <c r="M23" s="90" t="n"/>
-      <c r="N23" s="90" t="n"/>
-      <c r="O23" s="90" t="n"/>
-      <c r="P23" s="85" t="n"/>
-      <c r="Q23" s="85" t="n"/>
+      <c r="A23" s="85"/>
+      <c r="B23" s="86"/>
+      <c r="C23" s="86"/>
+      <c r="D23" s="86"/>
+      <c r="E23" s="86"/>
+      <c r="F23" s="87"/>
+      <c r="G23" s="85"/>
+      <c r="H23" s="88"/>
+      <c r="I23" s="88"/>
+      <c r="J23" s="88"/>
+      <c r="K23" s="88"/>
+      <c r="L23" s="89"/>
+      <c r="M23" s="90"/>
+      <c r="N23" s="90"/>
+      <c r="O23" s="90"/>
+      <c r="P23" s="85"/>
+      <c r="Q23" s="85"/>
     </row>
     <row r="24" ht="7.5" customHeight="1" s="50">
-      <c r="A24" s="85" t="n"/>
-      <c r="B24" s="87" t="n"/>
-      <c r="C24" s="87" t="n"/>
-      <c r="D24" s="87" t="n"/>
-      <c r="E24" s="87" t="n"/>
-      <c r="F24" s="86" t="n"/>
-      <c r="G24" s="85" t="n"/>
-      <c r="H24" s="88" t="n"/>
-      <c r="I24" s="88" t="n"/>
-      <c r="J24" s="88" t="n"/>
-      <c r="K24" s="88" t="n"/>
-      <c r="L24" s="89" t="n"/>
-      <c r="M24" s="90" t="n"/>
-      <c r="N24" s="90" t="n"/>
-      <c r="O24" s="90" t="n"/>
-      <c r="P24" s="85" t="n"/>
-      <c r="Q24" s="85" t="n"/>
+      <c r="A24" s="85"/>
+      <c r="B24" s="87"/>
+      <c r="C24" s="87"/>
+      <c r="D24" s="87"/>
+      <c r="E24" s="87"/>
+      <c r="F24" s="86"/>
+      <c r="G24" s="85"/>
+      <c r="H24" s="88"/>
+      <c r="I24" s="88"/>
+      <c r="J24" s="88"/>
+      <c r="K24" s="88"/>
+      <c r="L24" s="89"/>
+      <c r="M24" s="90"/>
+      <c r="N24" s="90"/>
+      <c r="O24" s="90"/>
+      <c r="P24" s="85"/>
+      <c r="Q24" s="85"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="50">
-      <c r="A25" s="86" t="n"/>
-      <c r="B25" s="86" t="n"/>
-      <c r="C25" s="86" t="n"/>
-      <c r="D25" s="86" t="n"/>
-      <c r="E25" s="86" t="n"/>
-      <c r="F25" s="87" t="n"/>
-      <c r="G25" s="86" t="n"/>
-      <c r="H25" s="91" t="n"/>
-      <c r="I25" s="91" t="n"/>
-      <c r="J25" s="91" t="n"/>
-      <c r="K25" s="91" t="n"/>
-      <c r="L25" s="92" t="n"/>
-      <c r="M25" s="93" t="n"/>
-      <c r="N25" s="93" t="n"/>
-      <c r="O25" s="93" t="n"/>
-      <c r="P25" s="86" t="n"/>
-      <c r="Q25" s="86" t="n"/>
+      <c r="A25" s="86"/>
+      <c r="B25" s="86"/>
+      <c r="C25" s="86"/>
+      <c r="D25" s="86"/>
+      <c r="E25" s="86"/>
+      <c r="F25" s="87"/>
+      <c r="G25" s="86"/>
+      <c r="H25" s="91"/>
+      <c r="I25" s="91"/>
+      <c r="J25" s="91"/>
+      <c r="K25" s="91"/>
+      <c r="L25" s="92"/>
+      <c r="M25" s="93"/>
+      <c r="N25" s="93"/>
+      <c r="O25" s="93"/>
+      <c r="P25" s="86"/>
+      <c r="Q25" s="86"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="50">
-      <c r="A26" s="94" t="n"/>
-      <c r="B26" s="94" t="n"/>
-      <c r="C26" s="94" t="n"/>
-      <c r="D26" s="94" t="n"/>
-      <c r="E26" s="94" t="n"/>
-      <c r="F26" s="94" t="n"/>
-      <c r="G26" s="87" t="n"/>
-      <c r="H26" s="99" t="n"/>
-      <c r="I26" s="99" t="n"/>
-      <c r="J26" s="99" t="n"/>
-      <c r="K26" s="99" t="n"/>
-      <c r="L26" s="96" t="n"/>
-      <c r="M26" s="97" t="n"/>
-      <c r="N26" s="97" t="n"/>
-      <c r="O26" s="97" t="n"/>
-      <c r="P26" s="98" t="n"/>
-      <c r="Q26" s="98" t="n"/>
+      <c r="A26" s="94"/>
+      <c r="B26" s="94"/>
+      <c r="C26" s="94"/>
+      <c r="D26" s="94"/>
+      <c r="E26" s="94"/>
+      <c r="F26" s="94"/>
+      <c r="G26" s="87"/>
+      <c r="H26" s="99"/>
+      <c r="I26" s="99"/>
+      <c r="J26" s="99"/>
+      <c r="K26" s="99"/>
+      <c r="L26" s="96"/>
+      <c r="M26" s="97"/>
+      <c r="N26" s="97"/>
+      <c r="O26" s="97"/>
+      <c r="P26" s="98"/>
+      <c r="Q26" s="98"/>
     </row>
     <row r="27" ht="7.5" customHeight="1" s="50">
-      <c r="A27" s="85" t="n"/>
-      <c r="B27" s="86" t="n"/>
-      <c r="C27" s="86" t="n"/>
-      <c r="D27" s="86" t="n"/>
-      <c r="E27" s="86" t="n"/>
-      <c r="F27" s="87" t="n"/>
-      <c r="G27" s="85" t="n"/>
-      <c r="H27" s="88" t="n"/>
-      <c r="I27" s="88" t="n"/>
-      <c r="J27" s="88" t="n"/>
-      <c r="K27" s="88" t="n"/>
-      <c r="L27" s="89" t="n"/>
-      <c r="M27" s="90" t="n"/>
-      <c r="N27" s="90" t="n"/>
-      <c r="O27" s="90" t="n"/>
-      <c r="P27" s="85" t="n"/>
-      <c r="Q27" s="85" t="n"/>
+      <c r="A27" s="85"/>
+      <c r="B27" s="86"/>
+      <c r="C27" s="86"/>
+      <c r="D27" s="86"/>
+      <c r="E27" s="86"/>
+      <c r="F27" s="87"/>
+      <c r="G27" s="85"/>
+      <c r="H27" s="88"/>
+      <c r="I27" s="88"/>
+      <c r="J27" s="88"/>
+      <c r="K27" s="88"/>
+      <c r="L27" s="89"/>
+      <c r="M27" s="90"/>
+      <c r="N27" s="90"/>
+      <c r="O27" s="90"/>
+      <c r="P27" s="85"/>
+      <c r="Q27" s="85"/>
     </row>
     <row r="28" ht="7.5" customHeight="1" s="50">
-      <c r="A28" s="85" t="n"/>
-      <c r="B28" s="87" t="n"/>
-      <c r="C28" s="87" t="n"/>
-      <c r="D28" s="87" t="n"/>
-      <c r="E28" s="87" t="n"/>
-      <c r="F28" s="86" t="n"/>
-      <c r="G28" s="85" t="n"/>
-      <c r="H28" s="88" t="n"/>
-      <c r="I28" s="88" t="n"/>
-      <c r="J28" s="88" t="n"/>
-      <c r="K28" s="88" t="n"/>
-      <c r="L28" s="89" t="n"/>
-      <c r="M28" s="90" t="n"/>
-      <c r="N28" s="90" t="n"/>
-      <c r="O28" s="90" t="n"/>
-      <c r="P28" s="85" t="n"/>
-      <c r="Q28" s="85" t="n"/>
+      <c r="A28" s="85"/>
+      <c r="B28" s="87"/>
+      <c r="C28" s="87"/>
+      <c r="D28" s="87"/>
+      <c r="E28" s="87"/>
+      <c r="F28" s="86"/>
+      <c r="G28" s="85"/>
+      <c r="H28" s="88"/>
+      <c r="I28" s="88"/>
+      <c r="J28" s="88"/>
+      <c r="K28" s="88"/>
+      <c r="L28" s="89"/>
+      <c r="M28" s="90"/>
+      <c r="N28" s="90"/>
+      <c r="O28" s="90"/>
+      <c r="P28" s="85"/>
+      <c r="Q28" s="85"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="50">
-      <c r="A29" s="86" t="n"/>
-      <c r="B29" s="86" t="n"/>
-      <c r="C29" s="86" t="n"/>
-      <c r="D29" s="86" t="n"/>
-      <c r="E29" s="86" t="n"/>
-      <c r="F29" s="87" t="n"/>
-      <c r="G29" s="86" t="n"/>
-      <c r="H29" s="91" t="n"/>
-      <c r="I29" s="91" t="n"/>
-      <c r="J29" s="91" t="n"/>
-      <c r="K29" s="91" t="n"/>
-      <c r="L29" s="92" t="n"/>
-      <c r="M29" s="93" t="n"/>
-      <c r="N29" s="93" t="n"/>
-      <c r="O29" s="93" t="n"/>
-      <c r="P29" s="86" t="n"/>
-      <c r="Q29" s="86" t="n"/>
+      <c r="A29" s="86"/>
+      <c r="B29" s="86"/>
+      <c r="C29" s="86"/>
+      <c r="D29" s="86"/>
+      <c r="E29" s="86"/>
+      <c r="F29" s="87"/>
+      <c r="G29" s="86"/>
+      <c r="H29" s="91"/>
+      <c r="I29" s="91"/>
+      <c r="J29" s="91"/>
+      <c r="K29" s="91"/>
+      <c r="L29" s="92"/>
+      <c r="M29" s="93"/>
+      <c r="N29" s="93"/>
+      <c r="O29" s="93"/>
+      <c r="P29" s="86"/>
+      <c r="Q29" s="86"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="50">
-      <c r="A30" s="94" t="n"/>
-      <c r="B30" s="94" t="n"/>
-      <c r="C30" s="94" t="n"/>
-      <c r="D30" s="94" t="n"/>
-      <c r="E30" s="94" t="n"/>
-      <c r="F30" s="94" t="n"/>
-      <c r="G30" s="87" t="n"/>
-      <c r="H30" s="99" t="n"/>
-      <c r="I30" s="99" t="n"/>
-      <c r="J30" s="99" t="n"/>
-      <c r="K30" s="99" t="n"/>
-      <c r="L30" s="96" t="n"/>
-      <c r="M30" s="97" t="n"/>
-      <c r="N30" s="97" t="n"/>
-      <c r="O30" s="97" t="n"/>
-      <c r="P30" s="98" t="n"/>
-      <c r="Q30" s="98" t="n"/>
+      <c r="A30" s="94"/>
+      <c r="B30" s="94"/>
+      <c r="C30" s="94"/>
+      <c r="D30" s="94"/>
+      <c r="E30" s="94"/>
+      <c r="F30" s="94"/>
+      <c r="G30" s="87"/>
+      <c r="H30" s="99"/>
+      <c r="I30" s="99"/>
+      <c r="J30" s="99"/>
+      <c r="K30" s="99"/>
+      <c r="L30" s="96"/>
+      <c r="M30" s="97"/>
+      <c r="N30" s="97"/>
+      <c r="O30" s="97"/>
+      <c r="P30" s="98"/>
+      <c r="Q30" s="98"/>
     </row>
     <row r="31" ht="7.5" customHeight="1" s="50">
-      <c r="A31" s="85" t="n"/>
-      <c r="B31" s="86" t="n"/>
-      <c r="C31" s="86" t="n"/>
-      <c r="D31" s="86" t="n"/>
-      <c r="E31" s="86" t="n"/>
-      <c r="F31" s="87" t="n"/>
-      <c r="G31" s="85" t="n"/>
-      <c r="H31" s="88" t="n"/>
-      <c r="I31" s="88" t="n"/>
-      <c r="J31" s="88" t="n"/>
-      <c r="K31" s="88" t="n"/>
-      <c r="L31" s="89" t="n"/>
-      <c r="M31" s="90" t="n"/>
-      <c r="N31" s="90" t="n"/>
-      <c r="O31" s="90" t="n"/>
-      <c r="P31" s="85" t="n"/>
-      <c r="Q31" s="85" t="n"/>
+      <c r="A31" s="85"/>
+      <c r="B31" s="86"/>
+      <c r="C31" s="86"/>
+      <c r="D31" s="86"/>
+      <c r="E31" s="86"/>
+      <c r="F31" s="87"/>
+      <c r="G31" s="85"/>
+      <c r="H31" s="88"/>
+      <c r="I31" s="88"/>
+      <c r="J31" s="88"/>
+      <c r="K31" s="88"/>
+      <c r="L31" s="89"/>
+      <c r="M31" s="90"/>
+      <c r="N31" s="90"/>
+      <c r="O31" s="90"/>
+      <c r="P31" s="85"/>
+      <c r="Q31" s="85"/>
     </row>
     <row r="32" ht="7.5" customHeight="1" s="50">
-      <c r="A32" s="85" t="n"/>
-      <c r="B32" s="87" t="n"/>
-      <c r="C32" s="87" t="n"/>
-      <c r="D32" s="87" t="n"/>
-      <c r="E32" s="87" t="n"/>
-      <c r="F32" s="86" t="n"/>
-      <c r="G32" s="85" t="n"/>
-      <c r="H32" s="88" t="n"/>
-      <c r="I32" s="88" t="n"/>
-      <c r="J32" s="88" t="n"/>
-      <c r="K32" s="88" t="n"/>
-      <c r="L32" s="89" t="n"/>
-      <c r="M32" s="90" t="n"/>
-      <c r="N32" s="90" t="n"/>
-      <c r="O32" s="90" t="n"/>
-      <c r="P32" s="85" t="n"/>
-      <c r="Q32" s="85" t="n"/>
+      <c r="A32" s="85"/>
+      <c r="B32" s="87"/>
+      <c r="C32" s="87"/>
+      <c r="D32" s="87"/>
+      <c r="E32" s="87"/>
+      <c r="F32" s="86"/>
+      <c r="G32" s="85"/>
+      <c r="H32" s="88"/>
+      <c r="I32" s="88"/>
+      <c r="J32" s="88"/>
+      <c r="K32" s="88"/>
+      <c r="L32" s="89"/>
+      <c r="M32" s="90"/>
+      <c r="N32" s="90"/>
+      <c r="O32" s="90"/>
+      <c r="P32" s="85"/>
+      <c r="Q32" s="85"/>
     </row>
     <row r="33" ht="15" customHeight="1" s="50">
-      <c r="A33" s="86" t="n"/>
-      <c r="B33" s="86" t="n"/>
-      <c r="C33" s="86" t="n"/>
-      <c r="D33" s="86" t="n"/>
-      <c r="E33" s="86" t="n"/>
-      <c r="F33" s="87" t="n"/>
-      <c r="G33" s="86" t="n"/>
-      <c r="H33" s="91" t="n"/>
-      <c r="I33" s="91" t="n"/>
-      <c r="J33" s="91" t="n"/>
-      <c r="K33" s="91" t="n"/>
-      <c r="L33" s="92" t="n"/>
-      <c r="M33" s="93" t="n"/>
-      <c r="N33" s="93" t="n"/>
-      <c r="O33" s="93" t="n"/>
-      <c r="P33" s="86" t="n"/>
-      <c r="Q33" s="86" t="n"/>
+      <c r="A33" s="86"/>
+      <c r="B33" s="86"/>
+      <c r="C33" s="86"/>
+      <c r="D33" s="86"/>
+      <c r="E33" s="86"/>
+      <c r="F33" s="87"/>
+      <c r="G33" s="86"/>
+      <c r="H33" s="91"/>
+      <c r="I33" s="91"/>
+      <c r="J33" s="91"/>
+      <c r="K33" s="91"/>
+      <c r="L33" s="92"/>
+      <c r="M33" s="93"/>
+      <c r="N33" s="93"/>
+      <c r="O33" s="93"/>
+      <c r="P33" s="86"/>
+      <c r="Q33" s="86"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="50">
-      <c r="A34" s="94" t="n"/>
-      <c r="B34" s="94" t="n"/>
-      <c r="C34" s="94" t="n"/>
-      <c r="D34" s="94" t="n"/>
-      <c r="E34" s="94" t="n"/>
-      <c r="F34" s="94" t="n"/>
-      <c r="G34" s="87" t="n"/>
-      <c r="H34" s="99" t="n"/>
-      <c r="I34" s="99" t="n"/>
-      <c r="J34" s="99" t="n"/>
-      <c r="K34" s="99" t="n"/>
-      <c r="L34" s="96" t="n"/>
-      <c r="M34" s="97" t="n"/>
-      <c r="N34" s="97" t="n"/>
-      <c r="O34" s="97" t="n"/>
-      <c r="P34" s="98" t="n"/>
-      <c r="Q34" s="98" t="n"/>
+      <c r="A34" s="94"/>
+      <c r="B34" s="94"/>
+      <c r="C34" s="94"/>
+      <c r="D34" s="94"/>
+      <c r="E34" s="94"/>
+      <c r="F34" s="94"/>
+      <c r="G34" s="87"/>
+      <c r="H34" s="99"/>
+      <c r="I34" s="99"/>
+      <c r="J34" s="99"/>
+      <c r="K34" s="99"/>
+      <c r="L34" s="96"/>
+      <c r="M34" s="97"/>
+      <c r="N34" s="97"/>
+      <c r="O34" s="97"/>
+      <c r="P34" s="98"/>
+      <c r="Q34" s="98"/>
     </row>
     <row r="35" ht="7.5" customHeight="1" s="50">
-      <c r="A35" s="85" t="n"/>
-      <c r="B35" s="86" t="n"/>
-      <c r="C35" s="86" t="n"/>
-      <c r="D35" s="86" t="n"/>
-      <c r="E35" s="86" t="n"/>
-      <c r="F35" s="87" t="n"/>
-      <c r="G35" s="85" t="n"/>
-      <c r="H35" s="88" t="n"/>
-      <c r="I35" s="88" t="n"/>
-      <c r="J35" s="88" t="n"/>
-      <c r="K35" s="88" t="n"/>
-      <c r="L35" s="89" t="n"/>
-      <c r="M35" s="90" t="n"/>
-      <c r="N35" s="90" t="n"/>
-      <c r="O35" s="90" t="n"/>
-      <c r="P35" s="85" t="n"/>
-      <c r="Q35" s="85" t="n"/>
+      <c r="A35" s="85"/>
+      <c r="B35" s="86"/>
+      <c r="C35" s="86"/>
+      <c r="D35" s="86"/>
+      <c r="E35" s="86"/>
+      <c r="F35" s="87"/>
+      <c r="G35" s="85"/>
+      <c r="H35" s="88"/>
+      <c r="I35" s="88"/>
+      <c r="J35" s="88"/>
+      <c r="K35" s="88"/>
+      <c r="L35" s="89"/>
+      <c r="M35" s="90"/>
+      <c r="N35" s="90"/>
+      <c r="O35" s="90"/>
+      <c r="P35" s="85"/>
+      <c r="Q35" s="85"/>
     </row>
     <row r="36" ht="7.5" customHeight="1" s="50">
-      <c r="A36" s="85" t="n"/>
-      <c r="B36" s="87" t="n"/>
-      <c r="C36" s="87" t="n"/>
-      <c r="D36" s="87" t="n"/>
-      <c r="E36" s="87" t="n"/>
-      <c r="F36" s="86" t="n"/>
-      <c r="G36" s="85" t="n"/>
-      <c r="H36" s="88" t="n"/>
-      <c r="I36" s="88" t="n"/>
-      <c r="J36" s="88" t="n"/>
-      <c r="K36" s="88" t="n"/>
-      <c r="L36" s="89" t="n"/>
-      <c r="M36" s="90" t="n"/>
-      <c r="N36" s="90" t="n"/>
-      <c r="O36" s="90" t="n"/>
-      <c r="P36" s="85" t="n"/>
-      <c r="Q36" s="85" t="n"/>
+      <c r="A36" s="85"/>
+      <c r="B36" s="87"/>
+      <c r="C36" s="87"/>
+      <c r="D36" s="87"/>
+      <c r="E36" s="87"/>
+      <c r="F36" s="86"/>
+      <c r="G36" s="85"/>
+      <c r="H36" s="88"/>
+      <c r="I36" s="88"/>
+      <c r="J36" s="88"/>
+      <c r="K36" s="88"/>
+      <c r="L36" s="89"/>
+      <c r="M36" s="90"/>
+      <c r="N36" s="90"/>
+      <c r="O36" s="90"/>
+      <c r="P36" s="85"/>
+      <c r="Q36" s="85"/>
     </row>
     <row r="37" ht="15" customHeight="1" s="50">
-      <c r="A37" s="86" t="n"/>
-      <c r="B37" s="86" t="n"/>
-      <c r="C37" s="86" t="n"/>
-      <c r="D37" s="86" t="n"/>
-      <c r="E37" s="86" t="n"/>
-      <c r="F37" s="87" t="n"/>
-      <c r="G37" s="86" t="n"/>
-      <c r="H37" s="91" t="n"/>
-      <c r="I37" s="91" t="n"/>
-      <c r="J37" s="91" t="n"/>
-      <c r="K37" s="91" t="n"/>
-      <c r="L37" s="92" t="n"/>
-      <c r="M37" s="93" t="n"/>
-      <c r="N37" s="93" t="n"/>
-      <c r="O37" s="93" t="n"/>
-      <c r="P37" s="86" t="n"/>
-      <c r="Q37" s="86" t="n"/>
+      <c r="A37" s="86"/>
+      <c r="B37" s="86"/>
+      <c r="C37" s="86"/>
+      <c r="D37" s="86"/>
+      <c r="E37" s="86"/>
+      <c r="F37" s="87"/>
+      <c r="G37" s="86"/>
+      <c r="H37" s="91"/>
+      <c r="I37" s="91"/>
+      <c r="J37" s="91"/>
+      <c r="K37" s="91"/>
+      <c r="L37" s="92"/>
+      <c r="M37" s="93"/>
+      <c r="N37" s="93"/>
+      <c r="O37" s="93"/>
+      <c r="P37" s="86"/>
+      <c r="Q37" s="86"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="50">
-      <c r="A38" s="94" t="n"/>
-      <c r="B38" s="94" t="n"/>
-      <c r="C38" s="94" t="n"/>
-      <c r="D38" s="94" t="n"/>
-      <c r="E38" s="94" t="n"/>
-      <c r="F38" s="94" t="n"/>
-      <c r="G38" s="87" t="n"/>
-      <c r="H38" s="99" t="n"/>
-      <c r="I38" s="99" t="n"/>
-      <c r="J38" s="99" t="n"/>
-      <c r="K38" s="99" t="n"/>
-      <c r="L38" s="96" t="n"/>
-      <c r="M38" s="97" t="n"/>
-      <c r="N38" s="97" t="n"/>
-      <c r="O38" s="97" t="n"/>
-      <c r="P38" s="98" t="n"/>
-      <c r="Q38" s="98" t="n"/>
+      <c r="A38" s="94"/>
+      <c r="B38" s="94"/>
+      <c r="C38" s="94"/>
+      <c r="D38" s="94"/>
+      <c r="E38" s="94"/>
+      <c r="F38" s="94"/>
+      <c r="G38" s="87"/>
+      <c r="H38" s="99"/>
+      <c r="I38" s="99"/>
+      <c r="J38" s="99"/>
+      <c r="K38" s="99"/>
+      <c r="L38" s="96"/>
+      <c r="M38" s="97"/>
+      <c r="N38" s="97"/>
+      <c r="O38" s="97"/>
+      <c r="P38" s="98"/>
+      <c r="Q38" s="98"/>
     </row>
     <row r="39" ht="7.5" customHeight="1" s="50">
-      <c r="A39" s="85" t="n"/>
-      <c r="B39" s="86" t="n"/>
-      <c r="C39" s="86" t="n"/>
-      <c r="D39" s="86" t="n"/>
-      <c r="E39" s="86" t="n"/>
-      <c r="F39" s="87" t="n"/>
-      <c r="G39" s="85" t="n"/>
-      <c r="H39" s="88" t="n"/>
-      <c r="I39" s="88" t="n"/>
-      <c r="J39" s="88" t="n"/>
-      <c r="K39" s="88" t="n"/>
-      <c r="L39" s="89" t="n"/>
-      <c r="M39" s="90" t="n"/>
-      <c r="N39" s="90" t="n"/>
-      <c r="O39" s="90" t="n"/>
-      <c r="P39" s="85" t="n"/>
-      <c r="Q39" s="85" t="n"/>
+      <c r="A39" s="85"/>
+      <c r="B39" s="86"/>
+      <c r="C39" s="86"/>
+      <c r="D39" s="86"/>
+      <c r="E39" s="86"/>
+      <c r="F39" s="87"/>
+      <c r="G39" s="85"/>
+      <c r="H39" s="88"/>
+      <c r="I39" s="88"/>
+      <c r="J39" s="88"/>
+      <c r="K39" s="88"/>
+      <c r="L39" s="89"/>
+      <c r="M39" s="90"/>
+      <c r="N39" s="90"/>
+      <c r="O39" s="90"/>
+      <c r="P39" s="85"/>
+      <c r="Q39" s="85"/>
     </row>
     <row r="40" ht="7.5" customHeight="1" s="50">
-      <c r="A40" s="85" t="n"/>
-      <c r="B40" s="87" t="n"/>
-      <c r="C40" s="87" t="n"/>
-      <c r="D40" s="87" t="n"/>
-      <c r="E40" s="87" t="n"/>
-      <c r="F40" s="86" t="n"/>
-      <c r="G40" s="85" t="n"/>
-      <c r="H40" s="88" t="n"/>
-      <c r="I40" s="88" t="n"/>
-      <c r="J40" s="88" t="n"/>
-      <c r="K40" s="88" t="n"/>
-      <c r="L40" s="89" t="n"/>
-      <c r="M40" s="90" t="n"/>
-      <c r="N40" s="90" t="n"/>
-      <c r="O40" s="90" t="n"/>
-      <c r="P40" s="85" t="n"/>
-      <c r="Q40" s="85" t="n"/>
+      <c r="A40" s="85"/>
+      <c r="B40" s="87"/>
+      <c r="C40" s="87"/>
+      <c r="D40" s="87"/>
+      <c r="E40" s="87"/>
+      <c r="F40" s="86"/>
+      <c r="G40" s="85"/>
+      <c r="H40" s="88"/>
+      <c r="I40" s="88"/>
+      <c r="J40" s="88"/>
+      <c r="K40" s="88"/>
+      <c r="L40" s="89"/>
+      <c r="M40" s="90"/>
+      <c r="N40" s="90"/>
+      <c r="O40" s="90"/>
+      <c r="P40" s="85"/>
+      <c r="Q40" s="85"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="50">
-      <c r="A41" s="86" t="n"/>
-      <c r="B41" s="86" t="n"/>
-      <c r="C41" s="86" t="n"/>
-      <c r="D41" s="86" t="n"/>
-      <c r="E41" s="86" t="n"/>
-      <c r="F41" s="87" t="n"/>
-      <c r="G41" s="86" t="n"/>
-      <c r="H41" s="91" t="n"/>
-      <c r="I41" s="91" t="n"/>
-      <c r="J41" s="91" t="n"/>
-      <c r="K41" s="91" t="n"/>
-      <c r="L41" s="92" t="n"/>
-      <c r="M41" s="93" t="n"/>
-      <c r="N41" s="93" t="n"/>
-      <c r="O41" s="93" t="n"/>
-      <c r="P41" s="86" t="n"/>
-      <c r="Q41" s="86" t="n"/>
+      <c r="A41" s="86"/>
+      <c r="B41" s="86"/>
+      <c r="C41" s="86"/>
+      <c r="D41" s="86"/>
+      <c r="E41" s="86"/>
+      <c r="F41" s="87"/>
+      <c r="G41" s="86"/>
+      <c r="H41" s="91"/>
+      <c r="I41" s="91"/>
+      <c r="J41" s="91"/>
+      <c r="K41" s="91"/>
+      <c r="L41" s="92"/>
+      <c r="M41" s="93"/>
+      <c r="N41" s="93"/>
+      <c r="O41" s="93"/>
+      <c r="P41" s="86"/>
+      <c r="Q41" s="86"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="50">
-      <c r="A42" s="100" t="n"/>
-      <c r="B42" s="100" t="n"/>
-      <c r="C42" s="100" t="n"/>
-      <c r="D42" s="100" t="n"/>
-      <c r="E42" s="100" t="n"/>
-      <c r="F42" s="100" t="n"/>
-      <c r="G42" s="100" t="n"/>
-      <c r="H42" s="100" t="n"/>
-      <c r="I42" s="100" t="n"/>
-      <c r="J42" s="100" t="n"/>
-      <c r="K42" s="100" t="n"/>
-      <c r="L42" s="100" t="n"/>
-      <c r="M42" s="100" t="n"/>
-      <c r="N42" s="100" t="n"/>
-      <c r="O42" s="100" t="n"/>
-      <c r="P42" s="49" t="n"/>
-      <c r="Q42" s="49" t="n"/>
+      <c r="A42" s="100"/>
+      <c r="B42" s="100"/>
+      <c r="C42" s="100"/>
+      <c r="D42" s="100"/>
+      <c r="E42" s="100"/>
+      <c r="F42" s="100"/>
+      <c r="G42" s="100"/>
+      <c r="H42" s="100"/>
+      <c r="I42" s="100"/>
+      <c r="J42" s="100"/>
+      <c r="K42" s="100"/>
+      <c r="L42" s="100"/>
+      <c r="M42" s="100"/>
+      <c r="N42" s="100"/>
+      <c r="O42" s="100"/>
+      <c r="P42" s="49"/>
+      <c r="Q42" s="49"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="50">
-      <c r="A43" s="100" t="n"/>
-      <c r="B43" s="100" t="n"/>
-      <c r="C43" s="100" t="n"/>
-      <c r="D43" s="100" t="n"/>
-      <c r="E43" s="100" t="n"/>
-      <c r="F43" s="100" t="n"/>
-      <c r="G43" s="100" t="n"/>
-      <c r="H43" s="100" t="n"/>
-      <c r="I43" s="100" t="n"/>
-      <c r="J43" s="100" t="n"/>
-      <c r="K43" s="100" t="n"/>
-      <c r="L43" s="100" t="n"/>
-      <c r="M43" s="100" t="n"/>
-      <c r="N43" s="100" t="n"/>
-      <c r="O43" s="100" t="n"/>
-      <c r="P43" s="49" t="n"/>
-      <c r="Q43" s="49" t="n"/>
+      <c r="A43" s="100"/>
+      <c r="B43" s="100"/>
+      <c r="C43" s="100"/>
+      <c r="D43" s="100"/>
+      <c r="E43" s="100"/>
+      <c r="F43" s="100"/>
+      <c r="G43" s="100"/>
+      <c r="H43" s="100"/>
+      <c r="I43" s="100"/>
+      <c r="J43" s="100"/>
+      <c r="K43" s="100"/>
+      <c r="L43" s="100"/>
+      <c r="M43" s="100"/>
+      <c r="N43" s="100"/>
+      <c r="O43" s="100"/>
+      <c r="P43" s="49"/>
+      <c r="Q43" s="49"/>
     </row>
     <row r="44" ht="14.4" customHeight="1" s="50">
       <c r="A44" s="101" t="s">
@@ -1701,392 +1701,185 @@
       <c r="B44" s="102" t="s">
         <v>26</v>
       </c>
-      <c r="C44" s="103" t="n"/>
-      <c r="D44" s="103" t="n"/>
-      <c r="E44" s="103" t="n"/>
-      <c r="F44" s="103" t="n"/>
-      <c r="G44" s="103" t="n"/>
-      <c r="H44" s="103" t="n"/>
-      <c r="I44" s="103" t="n"/>
-      <c r="J44" s="103" t="n"/>
-      <c r="K44" s="103" t="n"/>
-      <c r="L44" s="103" t="n"/>
-      <c r="M44" s="103" t="n"/>
-      <c r="N44" s="103" t="n"/>
-      <c r="O44" s="103" t="n"/>
-      <c r="P44" s="103" t="n"/>
-      <c r="Q44" s="103" t="n"/>
+      <c r="C44" s="103"/>
+      <c r="D44" s="103"/>
+      <c r="E44" s="103"/>
+      <c r="F44" s="103"/>
+      <c r="G44" s="103"/>
+      <c r="H44" s="103"/>
+      <c r="I44" s="103"/>
+      <c r="J44" s="103"/>
+      <c r="K44" s="103"/>
+      <c r="L44" s="103"/>
+      <c r="M44" s="103"/>
+      <c r="N44" s="103"/>
+      <c r="O44" s="103"/>
+      <c r="P44" s="103"/>
+      <c r="Q44" s="103"/>
     </row>
     <row r="45" ht="14.4" customHeight="1" s="50">
-      <c r="A45" s="102" t="n"/>
+      <c r="A45" s="102"/>
       <c r="B45" s="102" t="s">
         <v>27</v>
       </c>
-      <c r="C45" s="102" t="n"/>
-      <c r="D45" s="102" t="n"/>
-      <c r="E45" s="102" t="n"/>
-      <c r="F45" s="102" t="n"/>
-      <c r="G45" s="102" t="n"/>
-      <c r="H45" s="102" t="n"/>
-      <c r="I45" s="102" t="n"/>
-      <c r="J45" s="102" t="n"/>
-      <c r="K45" s="102" t="n"/>
-      <c r="L45" s="102" t="n"/>
-      <c r="M45" s="102" t="n"/>
-      <c r="N45" s="102" t="n"/>
-      <c r="O45" s="51" t="n"/>
-      <c r="P45" s="102" t="n"/>
-      <c r="Q45" s="102" t="n"/>
+      <c r="C45" s="102"/>
+      <c r="D45" s="102"/>
+      <c r="E45" s="102"/>
+      <c r="F45" s="102"/>
+      <c r="G45" s="102"/>
+      <c r="H45" s="102"/>
+      <c r="I45" s="102"/>
+      <c r="J45" s="102"/>
+      <c r="K45" s="102"/>
+      <c r="L45" s="102"/>
+      <c r="M45" s="102"/>
+      <c r="N45" s="102"/>
+      <c r="O45" s="51"/>
+      <c r="P45" s="102"/>
+      <c r="Q45" s="102"/>
     </row>
     <row r="46" ht="14.4" customHeight="1" s="50">
-      <c r="A46" s="102" t="n"/>
+      <c r="A46" s="102"/>
       <c r="B46" s="102" t="s">
         <v>28</v>
       </c>
-      <c r="C46" s="102" t="n"/>
-      <c r="D46" s="102" t="n"/>
-      <c r="E46" s="102" t="n"/>
-      <c r="F46" s="102" t="n"/>
-      <c r="G46" s="102" t="n"/>
-      <c r="H46" s="102" t="n"/>
-      <c r="I46" s="102" t="n"/>
-      <c r="J46" s="102" t="n"/>
-      <c r="K46" s="102" t="n"/>
-      <c r="L46" s="102" t="n"/>
-      <c r="M46" s="102" t="n"/>
-      <c r="N46" s="102" t="n"/>
-      <c r="O46" s="51" t="n"/>
-      <c r="P46" s="102" t="n"/>
-      <c r="Q46" s="102" t="n"/>
+      <c r="C46" s="102"/>
+      <c r="D46" s="102"/>
+      <c r="E46" s="102"/>
+      <c r="F46" s="102"/>
+      <c r="G46" s="102"/>
+      <c r="H46" s="102"/>
+      <c r="I46" s="102"/>
+      <c r="J46" s="102"/>
+      <c r="K46" s="102"/>
+      <c r="L46" s="102"/>
+      <c r="M46" s="102"/>
+      <c r="N46" s="102"/>
+      <c r="O46" s="51"/>
+      <c r="P46" s="102"/>
+      <c r="Q46" s="102"/>
     </row>
     <row r="47" ht="14.4" customHeight="1" s="50">
-      <c r="A47" s="102" t="n"/>
+      <c r="A47" s="102"/>
       <c r="B47" s="102" t="s">
         <v>29</v>
       </c>
-      <c r="C47" s="102" t="n"/>
-      <c r="D47" s="102" t="n"/>
-      <c r="E47" s="102" t="n"/>
-      <c r="F47" s="102" t="n"/>
-      <c r="G47" s="102" t="n"/>
-      <c r="H47" s="102" t="n"/>
-      <c r="I47" s="102" t="n"/>
-      <c r="J47" s="102" t="n"/>
-      <c r="K47" s="102" t="n"/>
-      <c r="L47" s="102" t="n"/>
-      <c r="M47" s="102" t="n"/>
-      <c r="N47" s="102" t="n"/>
-      <c r="O47" s="51" t="n"/>
-      <c r="P47" s="102" t="n"/>
-      <c r="Q47" s="102" t="n"/>
+      <c r="C47" s="102"/>
+      <c r="D47" s="102"/>
+      <c r="E47" s="102"/>
+      <c r="F47" s="102"/>
+      <c r="G47" s="102"/>
+      <c r="H47" s="102"/>
+      <c r="I47" s="102"/>
+      <c r="J47" s="102"/>
+      <c r="K47" s="102"/>
+      <c r="L47" s="102"/>
+      <c r="M47" s="102"/>
+      <c r="N47" s="102"/>
+      <c r="O47" s="51"/>
+      <c r="P47" s="102"/>
+      <c r="Q47" s="102"/>
     </row>
     <row r="48" ht="14.4" customHeight="1" s="50">
-      <c r="A48" s="103" t="n"/>
-      <c r="B48" s="103" t="n"/>
-      <c r="C48" s="103" t="n"/>
-      <c r="D48" s="103" t="n"/>
-      <c r="E48" s="103" t="n"/>
-      <c r="F48" s="49" t="n"/>
-      <c r="G48" s="49" t="n"/>
-      <c r="H48" s="103" t="n"/>
-      <c r="I48" s="103" t="n"/>
-      <c r="J48" s="49" t="n"/>
-      <c r="K48" s="103" t="n"/>
-      <c r="L48" s="103" t="n"/>
-      <c r="M48" s="103" t="n"/>
-      <c r="N48" s="103" t="n"/>
-      <c r="O48" s="103" t="n"/>
-      <c r="P48" s="49" t="n"/>
+      <c r="A48" s="103"/>
+      <c r="B48" s="103"/>
+      <c r="C48" s="103"/>
+      <c r="D48" s="103"/>
+      <c r="E48" s="103"/>
+      <c r="F48" s="49"/>
+      <c r="G48" s="49"/>
+      <c r="H48" s="103"/>
+      <c r="I48" s="103"/>
+      <c r="J48" s="49"/>
+      <c r="K48" s="103"/>
+      <c r="L48" s="103"/>
+      <c r="M48" s="103"/>
+      <c r="N48" s="103"/>
+      <c r="O48" s="103"/>
+      <c r="P48" s="49"/>
     </row>
     <row r="49" ht="14.4" customHeight="1" s="50">
-      <c r="A49" s="103" t="n"/>
+      <c r="A49" s="103"/>
       <c r="B49" s="103" t="s">
         <v>30</v>
       </c>
-      <c r="C49" s="103" t="n"/>
-      <c r="D49" s="103" t="n"/>
-      <c r="E49" s="103" t="n"/>
-      <c r="F49" s="103" t="n"/>
+      <c r="C49" s="103"/>
+      <c r="D49" s="103"/>
+      <c r="E49" s="103"/>
+      <c r="F49" s="103"/>
       <c r="G49" s="103" t="s">
         <v>31</v>
       </c>
-      <c r="H49" s="103" t="n"/>
-      <c r="I49" s="103" t="n"/>
-      <c r="J49" s="103" t="n"/>
+      <c r="H49" s="103"/>
+      <c r="I49" s="103"/>
+      <c r="J49" s="103"/>
       <c r="K49" s="103" t="s">
         <v>32</v>
       </c>
-      <c r="L49" s="103" t="n"/>
-      <c r="M49" s="103" t="n"/>
+      <c r="L49" s="103"/>
+      <c r="M49" s="103"/>
       <c r="N49" s="103" t="s">
         <v>33</v>
       </c>
-      <c r="O49" s="103" t="n"/>
-      <c r="P49" s="103" t="n"/>
-      <c r="Q49" s="103" t="n"/>
+      <c r="O49" s="103"/>
+      <c r="P49" s="103"/>
+      <c r="Q49" s="103"/>
     </row>
     <row r="50" ht="14.4" customHeight="1" s="50">
-      <c r="N50" s="49" t="n"/>
-      <c r="O50" s="104" t="n"/>
-      <c r="P50" s="104" t="n"/>
-      <c r="Q50" s="104" t="n"/>
+      <c r="N50" s="49"/>
+      <c r="O50" s="104"/>
+      <c r="P50" s="104"/>
+      <c r="Q50" s="104"/>
     </row>
     <row r="51" ht="14.4" customFormat="1" customHeight="1" s="57">
-      <c r="N51" s="104" t="n"/>
-      <c r="O51" s="104" t="n"/>
-      <c r="P51" s="104" t="n"/>
-      <c r="Q51" s="104" t="n"/>
+      <c r="N51" s="104"/>
+      <c r="O51" s="104"/>
+      <c r="P51" s="104"/>
+      <c r="Q51" s="104"/>
     </row>
     <row r="52" ht="14.4" customFormat="1" customHeight="1" s="57">
-      <c r="N52" s="104" t="n"/>
-      <c r="O52" s="104" t="n"/>
-      <c r="P52" s="104" t="n"/>
-      <c r="Q52" s="104" t="n"/>
+      <c r="N52" s="104"/>
+      <c r="O52" s="104"/>
+      <c r="P52" s="104"/>
+      <c r="Q52" s="104"/>
     </row>
     <row r="53" ht="14.4" customFormat="1" customHeight="1" s="57">
-      <c r="A53" s="102" t="n"/>
-      <c r="B53" s="102" t="n"/>
-      <c r="F53" s="102" t="n"/>
-      <c r="G53" s="102" t="n"/>
-      <c r="J53" s="102" t="n"/>
-      <c r="K53" s="102" t="n"/>
-      <c r="N53" s="102" t="n"/>
-      <c r="Q53" s="102" t="n"/>
+      <c r="A53" s="102"/>
+      <c r="B53" s="102"/>
+      <c r="F53" s="102"/>
+      <c r="G53" s="102"/>
+      <c r="J53" s="102"/>
+      <c r="K53" s="102"/>
+      <c r="N53" s="102"/>
+      <c r="Q53" s="102"/>
     </row>
     <row r="54" ht="13.8" customHeight="1" s="50">
-      <c r="A54" s="105" t="n"/>
+      <c r="A54" s="105"/>
       <c r="B54" s="105" t="s">
         <v>34</v>
       </c>
-      <c r="C54" s="105" t="n"/>
-      <c r="D54" s="105" t="n"/>
-      <c r="E54" s="105" t="n"/>
-      <c r="F54" s="105" t="n"/>
+      <c r="C54" s="105"/>
+      <c r="D54" s="105"/>
+      <c r="E54" s="105"/>
+      <c r="F54" s="105"/>
       <c r="G54" s="105" t="s">
         <v>35</v>
       </c>
-      <c r="H54" s="105" t="n"/>
-      <c r="I54" s="105" t="n"/>
-      <c r="J54" s="105" t="n"/>
+      <c r="H54" s="105"/>
+      <c r="I54" s="105"/>
+      <c r="J54" s="105"/>
       <c r="K54" s="105" t="s">
         <v>36</v>
       </c>
-      <c r="L54" s="105" t="n"/>
-      <c r="M54" s="105" t="n"/>
+      <c r="L54" s="105"/>
+      <c r="M54" s="105"/>
       <c r="N54" s="105" t="s">
         <v>37</v>
       </c>
-      <c r="O54" s="105" t="n"/>
-      <c r="P54" s="105" t="n"/>
-      <c r="Q54" s="105" t="n"/>
-    </row>
-    <row r="55" ht="27.75" customFormat="1" customHeight="1" s="63"/>
-    <row r="56" ht="16.5" customFormat="1" customHeight="1" s="63"/>
-    <row r="57" ht="15" customHeight="1" s="50"/>
-    <row r="58" ht="7.5" customHeight="1" s="50"/>
-    <row r="59" ht="7.5" customHeight="1" s="50"/>
-    <row r="60" ht="15" customHeight="1" s="50"/>
-    <row r="61" ht="15" customHeight="1" s="50"/>
-    <row r="62" ht="7.5" customHeight="1" s="50"/>
-    <row r="63" ht="7.5" customHeight="1" s="50"/>
-    <row r="64" ht="15" customHeight="1" s="50"/>
-    <row r="65" ht="15" customHeight="1" s="50"/>
-    <row r="66" ht="7.5" customHeight="1" s="50"/>
-    <row r="67" ht="7.5" customHeight="1" s="50"/>
-    <row r="68" ht="15" customHeight="1" s="50"/>
-    <row r="69" ht="15" customHeight="1" s="50"/>
-    <row r="70" ht="7.5" customHeight="1" s="50"/>
-    <row r="71" ht="7.5" customHeight="1" s="50"/>
-    <row r="72" ht="15" customHeight="1" s="50"/>
-    <row r="73" ht="15" customHeight="1" s="50"/>
-    <row r="74" ht="7.5" customHeight="1" s="50"/>
-    <row r="75" ht="7.5" customHeight="1" s="50"/>
-    <row r="76" ht="15" customHeight="1" s="50"/>
-    <row r="77" ht="15" customHeight="1" s="50"/>
-    <row r="78" ht="7.5" customHeight="1" s="50"/>
-    <row r="79" ht="7.5" customHeight="1" s="50"/>
-    <row r="80" ht="15" customHeight="1" s="50"/>
-    <row r="81" ht="15" customHeight="1" s="50"/>
-    <row r="82" ht="7.5" customHeight="1" s="50"/>
-    <row r="83" ht="7.5" customHeight="1" s="50"/>
-    <row r="84" ht="15" customHeight="1" s="50"/>
-    <row r="85" ht="15" customHeight="1" s="50"/>
-    <row r="86" ht="15" customHeight="1" s="50"/>
-    <row r="87" ht="14.4" customHeight="1" s="50"/>
-    <row r="88" ht="14.4" customHeight="1" s="50"/>
-    <row r="89" ht="14.4" customHeight="1" s="50"/>
-    <row r="90" ht="14.4" customHeight="1" s="50"/>
-    <row r="92" ht="18" customHeight="1" s="50"/>
-    <row r="94" ht="14.4" customFormat="1" customHeight="1" s="57"/>
-    <row r="95" ht="14.4" customFormat="1" customHeight="1" s="57"/>
-    <row r="96" ht="14.4" customFormat="1" customHeight="1" s="57"/>
-    <row r="97" ht="14.4" customHeight="1" s="50"/>
-    <row r="98" ht="27.75" customFormat="1" customHeight="1" s="63"/>
-    <row r="99" ht="16.5" customFormat="1" customHeight="1" s="63"/>
-    <row r="100" ht="15" customHeight="1" s="50"/>
-    <row r="101" ht="7.5" customHeight="1" s="50"/>
-    <row r="102" ht="7.5" customHeight="1" s="50"/>
-    <row r="103" ht="15" customHeight="1" s="50"/>
-    <row r="104" ht="15" customHeight="1" s="50"/>
-    <row r="105" ht="7.5" customHeight="1" s="50"/>
-    <row r="106" ht="7.5" customHeight="1" s="50"/>
-    <row r="107" ht="15" customHeight="1" s="50"/>
-    <row r="108" ht="15" customHeight="1" s="50"/>
-    <row r="109" ht="7.5" customHeight="1" s="50"/>
-    <row r="110" ht="7.5" customHeight="1" s="50"/>
-    <row r="111" ht="15" customHeight="1" s="50"/>
-    <row r="112" ht="15" customHeight="1" s="50"/>
-    <row r="113" ht="7.5" customHeight="1" s="50"/>
-    <row r="114" ht="7.5" customHeight="1" s="50"/>
-    <row r="115" ht="15" customHeight="1" s="50"/>
-    <row r="116" ht="15" customHeight="1" s="50"/>
-    <row r="117" ht="7.5" customHeight="1" s="50"/>
-    <row r="118" ht="7.5" customHeight="1" s="50"/>
-    <row r="119" ht="15" customHeight="1" s="50"/>
-    <row r="120" ht="15" customHeight="1" s="50"/>
-    <row r="121" ht="7.5" customHeight="1" s="50"/>
-    <row r="122" ht="7.5" customHeight="1" s="50"/>
-    <row r="123" ht="15" customHeight="1" s="50"/>
-    <row r="124" ht="15" customHeight="1" s="50"/>
-    <row r="125" ht="7.5" customHeight="1" s="50"/>
-    <row r="126" ht="7.5" customHeight="1" s="50"/>
-    <row r="127" ht="15" customHeight="1" s="50"/>
-    <row r="128" ht="15" customHeight="1" s="50"/>
-    <row r="129" ht="15" customHeight="1" s="50"/>
-    <row r="130" ht="14.4" customHeight="1" s="50"/>
-    <row r="131" ht="14.4" customHeight="1" s="50"/>
-    <row r="132" ht="14.4" customHeight="1" s="50"/>
-    <row r="133" ht="14.4" customHeight="1" s="50"/>
-    <row r="135" ht="18" customHeight="1" s="50"/>
-    <row r="137" ht="14.4" customFormat="1" customHeight="1" s="57"/>
-    <row r="138" ht="14.4" customFormat="1" customHeight="1" s="57"/>
-    <row r="139" ht="14.4" customFormat="1" customHeight="1" s="57"/>
-    <row r="140" ht="14.4" customHeight="1" s="50"/>
-    <row r="141" ht="27.75" customFormat="1" customHeight="1" s="63"/>
-    <row r="142" ht="16.5" customFormat="1" customHeight="1" s="63"/>
-    <row r="143" ht="15" customHeight="1" s="50"/>
-    <row r="144" ht="7.5" customHeight="1" s="50"/>
-    <row r="145" ht="7.5" customHeight="1" s="50"/>
-    <row r="146" ht="15" customHeight="1" s="50"/>
-    <row r="147" ht="15" customHeight="1" s="50"/>
-    <row r="148" ht="7.5" customHeight="1" s="50"/>
-    <row r="149" ht="7.5" customHeight="1" s="50"/>
-    <row r="150" ht="15" customHeight="1" s="50"/>
-    <row r="151" ht="15" customHeight="1" s="50"/>
-    <row r="152" ht="7.5" customHeight="1" s="50"/>
-    <row r="153" ht="7.5" customHeight="1" s="50"/>
-    <row r="154" ht="15" customHeight="1" s="50"/>
-    <row r="155" ht="15" customHeight="1" s="50"/>
-    <row r="156" ht="7.5" customHeight="1" s="50"/>
-    <row r="157" ht="7.5" customHeight="1" s="50"/>
-    <row r="158" ht="15" customHeight="1" s="50"/>
-    <row r="159" ht="15" customHeight="1" s="50"/>
-    <row r="160" ht="7.5" customHeight="1" s="50"/>
-    <row r="161" ht="7.5" customHeight="1" s="50"/>
-    <row r="162" ht="15" customHeight="1" s="50"/>
-    <row r="163" ht="15" customHeight="1" s="50"/>
-    <row r="164" ht="7.5" customHeight="1" s="50"/>
-    <row r="165" ht="7.5" customHeight="1" s="50"/>
-    <row r="166" ht="15" customHeight="1" s="50"/>
-    <row r="167" ht="15" customHeight="1" s="50"/>
-    <row r="168" ht="7.5" customHeight="1" s="50"/>
-    <row r="169" ht="7.5" customHeight="1" s="50"/>
-    <row r="170" ht="15" customHeight="1" s="50"/>
-    <row r="171" ht="15" customHeight="1" s="50"/>
-    <row r="172" ht="15" customHeight="1" s="50"/>
-    <row r="173" ht="14.4" customHeight="1" s="50"/>
-    <row r="174" ht="14.4" customHeight="1" s="50"/>
-    <row r="175" ht="14.4" customHeight="1" s="50"/>
-    <row r="176" ht="14.4" customHeight="1" s="50"/>
-    <row r="178" ht="18" customHeight="1" s="50"/>
-    <row r="180" ht="14.4" customFormat="1" customHeight="1" s="57"/>
-    <row r="181" ht="14.4" customFormat="1" customHeight="1" s="57"/>
-    <row r="182" ht="14.4" customFormat="1" customHeight="1" s="57"/>
-    <row r="183" ht="14.4" customHeight="1" s="50"/>
-    <row r="184" ht="27.75" customFormat="1" customHeight="1" s="63"/>
-    <row r="185" ht="16.5" customFormat="1" customHeight="1" s="63"/>
-    <row r="186" ht="15" customHeight="1" s="50"/>
-    <row r="187" ht="7.5" customHeight="1" s="50"/>
-    <row r="188" ht="7.5" customHeight="1" s="50"/>
-    <row r="189" ht="15" customHeight="1" s="50"/>
-    <row r="190" ht="15" customHeight="1" s="50"/>
-    <row r="191" ht="7.5" customHeight="1" s="50"/>
-    <row r="192" ht="7.5" customHeight="1" s="50"/>
-    <row r="193" ht="15" customHeight="1" s="50"/>
-    <row r="194" ht="15" customHeight="1" s="50"/>
-    <row r="195" ht="7.5" customHeight="1" s="50"/>
-    <row r="196" ht="7.5" customHeight="1" s="50"/>
-    <row r="197" ht="15" customHeight="1" s="50"/>
-    <row r="198" ht="15" customHeight="1" s="50"/>
-    <row r="199" ht="7.5" customHeight="1" s="50"/>
-    <row r="200" ht="7.5" customHeight="1" s="50"/>
-    <row r="201" ht="15" customHeight="1" s="50"/>
-    <row r="202" ht="15" customHeight="1" s="50"/>
-    <row r="203" ht="7.5" customHeight="1" s="50"/>
-    <row r="204" ht="7.5" customHeight="1" s="50"/>
-    <row r="205" ht="15" customHeight="1" s="50"/>
-    <row r="206" ht="15" customHeight="1" s="50"/>
-    <row r="207" ht="7.5" customHeight="1" s="50"/>
-    <row r="208" ht="7.5" customHeight="1" s="50"/>
-    <row r="209" ht="15" customHeight="1" s="50"/>
-    <row r="210" ht="15" customHeight="1" s="50"/>
-    <row r="211" ht="7.5" customHeight="1" s="50"/>
-    <row r="212" ht="7.5" customHeight="1" s="50"/>
-    <row r="213" ht="15" customHeight="1" s="50"/>
-    <row r="214" ht="15" customHeight="1" s="50"/>
-    <row r="215" ht="6.9" customHeight="1" s="50"/>
-    <row r="216" ht="13.8" customFormat="1" customHeight="1" s="103"/>
-    <row r="217" ht="13.8" customFormat="1" customHeight="1" s="102"/>
-    <row r="218" ht="13.8" customFormat="1" customHeight="1" s="102"/>
-    <row r="219" ht="13.8" customFormat="1" customHeight="1" s="102"/>
-    <row r="221" ht="18" customFormat="1" customHeight="1" s="103"/>
-    <row r="223" ht="14.4" customHeight="1" s="50"/>
-    <row r="224" ht="14.4" customHeight="1" s="50"/>
-    <row r="225" ht="14.4" customFormat="1" customHeight="1" s="102"/>
-    <row r="226" ht="14.4" customFormat="1" customHeight="1" s="105"/>
-    <row r="227" ht="14.4" customHeight="1" s="50"/>
-    <row r="228" ht="14.4" customHeight="1" s="50"/>
-    <row r="229" ht="14.4" customHeight="1" s="50"/>
-    <row r="230" ht="13.8" customHeight="1" s="50"/>
-    <row r="231" ht="13.8" customHeight="1" s="50"/>
-    <row r="232" ht="13.8" customHeight="1" s="50"/>
-    <row r="233" ht="13.8" customHeight="1" s="50"/>
-    <row r="234" ht="13.8" customHeight="1" s="50"/>
-    <row r="235" ht="13.8" customHeight="1" s="50"/>
-    <row r="236" ht="13.8" customHeight="1" s="50"/>
-    <row r="237" ht="13.8" customHeight="1" s="50"/>
-    <row r="238" ht="13.8" customHeight="1" s="50"/>
-    <row r="239" ht="13.8" customHeight="1" s="50"/>
-    <row r="240" ht="13.8" customHeight="1" s="50"/>
-    <row r="241" ht="13.8" customHeight="1" s="50"/>
-    <row r="242" ht="13.8" customHeight="1" s="50"/>
-    <row r="243" ht="13.8" customHeight="1" s="50"/>
-    <row r="244" ht="13.8" customHeight="1" s="50"/>
-    <row r="245" ht="13.8" customHeight="1" s="50"/>
-    <row r="246" ht="13.8" customHeight="1" s="50"/>
-    <row r="247" ht="13.8" customHeight="1" s="50"/>
-    <row r="248" ht="13.8" customHeight="1" s="50"/>
-    <row r="249" ht="13.8" customHeight="1" s="50"/>
-    <row r="250" ht="13.8" customHeight="1" s="50"/>
-    <row r="251" ht="13.8" customHeight="1" s="50"/>
-    <row r="252" ht="13.8" customHeight="1" s="50"/>
-    <row r="253" ht="13.8" customHeight="1" s="50"/>
-    <row r="254" ht="13.8" customHeight="1" s="50"/>
-    <row r="255" ht="13.8" customHeight="1" s="50"/>
-    <row r="256" ht="13.8" customHeight="1" s="50"/>
-    <row r="257" ht="14.4" customHeight="1" s="50"/>
-    <row r="258" ht="7.2" customHeight="1" s="50"/>
-    <row r="259" ht="14.4" customHeight="1" s="50"/>
-    <row r="260" ht="14.4" customHeight="1" s="50"/>
-    <row r="261" ht="14.4" customHeight="1" s="50"/>
-    <row r="262" ht="14.4" customHeight="1" s="50"/>
-    <row r="263" ht="14.4" customHeight="1" s="50"/>
-    <row r="264" ht="14.4" customHeight="1" s="50"/>
-    <row r="265" ht="14.4" customHeight="1" s="50"/>
-    <row r="266" ht="14.4" customHeight="1" s="50"/>
-    <row r="267" ht="14.4" customHeight="1" s="50"/>
-    <row r="268" ht="14.4" customHeight="1" s="50"/>
-    <row r="269" ht="13.8" customHeight="1" s="50"/>
+      <c r="O54" s="105"/>
+      <c r="P54" s="105"/>
+      <c r="Q54" s="105"/>
+    </row>
   </sheetData>
   <mergeCells count="152">
     <mergeCell ref="L18:O21"/>
@@ -2244,7 +2037,7 @@
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="5" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="landscape" paperSize="5" scale="100" fitToHeight="0" fitToWidth="0" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
     <oddFooter>&amp;L&amp;7 CC: PH. TRAMS / C B T.  OOD.  MSSD.  STATION  _x000a_Tel. 928-6683 Telfax. 920-6682 Ref. no. CCDR-061512/tdc-RMLJ</oddFooter>

</xml_diff>